<commit_message>
Add functionality to generate Excel reports by section
- Implemented functions to retrieve question sections and questions by section.
- Updated `run_report.py` to generate reports for each section.
- Enhanced `build_question_report` to handle multiple dataframes in a single Excel sheet.
</commit_message>
<xml_diff>
--- a/output/ocupacion.xlsx
+++ b/output/ocupacion.xlsx
@@ -7,8 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Principal ocupacion" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Modalidad" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Quehaceres" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -426,257 +425,820 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:N31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Respuesta por unidad geográfica</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>id_respuesta</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>Respuesta</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Hombre</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Mujer</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Empleado(a)</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>1123461.611426135</v>
-      </c>
-      <c r="D2" t="n">
-        <v>493096.3555596098</v>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Monterrey</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Guadalupe</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>San Nicolás de los Garza</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>Apodaca</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>Escobedo</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>San Pedro Garza García</t>
+        </is>
+      </c>
+      <c r="I2" s="1" t="inlineStr">
+        <is>
+          <t>Santiago</t>
+        </is>
+      </c>
+      <c r="J2" s="1" t="inlineStr">
+        <is>
+          <t>Juárez</t>
+        </is>
+      </c>
+      <c r="K2" s="1" t="inlineStr">
+        <is>
+          <t>García</t>
+        </is>
+      </c>
+      <c r="L2" s="1" t="inlineStr">
+        <is>
+          <t>Santa Catarina</t>
+        </is>
+      </c>
+      <c r="M2" s="1" t="inlineStr">
+        <is>
+          <t>Cadereyta</t>
+        </is>
+      </c>
+      <c r="N2" s="1" t="inlineStr">
+        <is>
+          <t>Resto NL</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Buscando empleo</t>
+          <t>Usted principalmente</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>150746.2942226993</v>
+        <v>326856.1107376305</v>
       </c>
       <c r="D3" t="n">
-        <v>49830.98440873342</v>
+        <v>178814.3907173525</v>
+      </c>
+      <c r="E3" t="n">
+        <v>139264.933435787</v>
+      </c>
+      <c r="F3" t="n">
+        <v>184157.2840142484</v>
+      </c>
+      <c r="G3" t="n">
+        <v>153735.8027421758</v>
+      </c>
+      <c r="H3" t="n">
+        <v>37099.16135825786</v>
+      </c>
+      <c r="I3" t="n">
+        <v>17013.48039193717</v>
+      </c>
+      <c r="J3" t="n">
+        <v>152438.7161078384</v>
+      </c>
+      <c r="K3" t="n">
+        <v>128243.6066560035</v>
+      </c>
+      <c r="L3" t="n">
+        <v>92225.28416259996</v>
+      </c>
+      <c r="M3" t="n">
+        <v>41619.00020623116</v>
+      </c>
+      <c r="N3" t="n">
+        <v>291787.7541275433</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Estudiante</t>
+          <t>Usted y otra(s) persona(s) del hogar por igual</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>120172.6416120934</v>
+        <v>374063.9345116179</v>
       </c>
       <c r="D4" t="n">
-        <v>97819.52766988361</v>
+        <v>245590.8278943268</v>
+      </c>
+      <c r="E4" t="n">
+        <v>147538.5930084813</v>
+      </c>
+      <c r="F4" t="n">
+        <v>265301.3491282744</v>
+      </c>
+      <c r="G4" t="n">
+        <v>135182.2900959865</v>
+      </c>
+      <c r="H4" t="n">
+        <v>34395.25129367346</v>
+      </c>
+      <c r="I4" t="n">
+        <v>14571.07048489924</v>
+      </c>
+      <c r="J4" t="n">
+        <v>144163.3241389042</v>
+      </c>
+      <c r="K4" t="n">
+        <v>110778.3427612085</v>
+      </c>
+      <c r="L4" t="n">
+        <v>113640.1037708144</v>
+      </c>
+      <c r="M4" t="n">
+        <v>31804.7250631487</v>
+      </c>
+      <c r="N4" t="n">
+        <v>310238.5929203792</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Negocio propio / independiente</t>
+          <t>Otro(a) miembro del hogar</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>430742.4544354618</v>
+        <v>184099.703926429</v>
       </c>
       <c r="D5" t="n">
-        <v>217172.4930031824</v>
+        <v>101960.1579200956</v>
+      </c>
+      <c r="E5" t="n">
+        <v>61793.13465877515</v>
+      </c>
+      <c r="F5" t="n">
+        <v>57490.00914223125</v>
+      </c>
+      <c r="G5" t="n">
+        <v>78782.08512053778</v>
+      </c>
+      <c r="H5" t="n">
+        <v>10206.40875807292</v>
+      </c>
+      <c r="I5" t="n">
+        <v>5430.458673901116</v>
+      </c>
+      <c r="J5" t="n">
+        <v>52856.08807142136</v>
+      </c>
+      <c r="K5" t="n">
+        <v>45661.88071597183</v>
+      </c>
+      <c r="L5" t="n">
+        <v>33741.57299504205</v>
+      </c>
+      <c r="M5" t="n">
+        <v>21060.02016510105</v>
+      </c>
+      <c r="N5" t="n">
+        <v>118129.3615169688</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Trabajo del hogar no remunerado (como limpiar la casa y cuidar niños o personas enfermas)</t>
+          <t>Una persona contratada (vive o no en el hogar)</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>27501.35207931548</v>
+        <v>59111.92274913648</v>
       </c>
       <c r="D6" t="n">
-        <v>1267187.358692795</v>
+        <v>6322.718670153653</v>
+      </c>
+      <c r="E6" t="n">
+        <v>6128.338896956896</v>
+      </c>
+      <c r="F6" t="n">
+        <v>6398.357715246018</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2535.053751641985</v>
+      </c>
+      <c r="H6" t="n">
+        <v>29961.55351529385</v>
+      </c>
+      <c r="I6" t="n">
+        <v>644.5271204514029</v>
+      </c>
+      <c r="J6" t="n">
+        <v>451.8716818358949</v>
+      </c>
+      <c r="K6" t="n">
+        <v>2130.169866816107</v>
+      </c>
+      <c r="L6" t="n">
+        <v>4690.039071543542</v>
+      </c>
+      <c r="M6" t="n">
+        <v>869.9055447013177</v>
+      </c>
+      <c r="N6" t="n">
+        <v>9768.291435108506</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Trabajo del hogar remunerado (limpieza de otros hogares)</t>
+          <t>Usted, con ayuda de una persona contratada uno o más días a la semana</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>465.6997232605394</v>
+        <v>1913.825517078612</v>
       </c>
       <c r="D7" t="n">
-        <v>12427.6272565119</v>
+        <v>822.9047980725754</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>603.7682896574496</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1689.18724376578</v>
+      </c>
+      <c r="I7" t="n">
+        <v>215.6885798028476</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="n">
+        <v>166.3490208176711</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Jubilado/Pensionado</t>
+          <t>Otro miembro del hogar, con ayuda de una persona contratada uno o más días a la semana</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>350551.1374219133</v>
+        <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>113079.7627395945</v>
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>198.437830935967</v>
+      </c>
+      <c r="I8" t="n">
+        <v>280.7747490082377</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>8</v>
+        <v>9999</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Ni estudia, ni trabaja, ni busca empleo</t>
+          <t>No contesta</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>68704.96531157823</v>
+        <v>5335.502558106416</v>
       </c>
       <c r="D9" t="n">
-        <v>48069.8541911649</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Respuesta por sexo</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>id_respuesta</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>Respuesta</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>Hombre</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>Mujer</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Usted principalmente</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>389053.8231383966</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1354201.701519209</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>2</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Usted y otra(s) persona(s) del hogar por igual</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1130882.858584785</v>
+      </c>
+      <c r="D15" t="n">
+        <v>796385.5464869295</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Otro(a) miembro del hogar</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>689183.9411531677</v>
+      </c>
+      <c r="D16" t="n">
+        <v>82026.94051138002</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>4</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Una persona contratada (vive o no en el hogar)</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>69633.72167246207</v>
+      </c>
+      <c r="D17" t="n">
+        <v>59379.02834642358</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>5</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Usted, con ayuda de una persona contratada uno o más días a la semana</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>1644.442871243648</v>
+      </c>
+      <c r="D18" t="n">
+        <v>3767.280577951287</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>6</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Otro miembro del hogar, con ayuda de una persona contratada uno o más días a la semana</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>479.2125799442047</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
         <v>9999</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>No contesta</t>
         </is>
       </c>
-      <c r="C10" t="n">
-        <v>8531.843767542448</v>
-      </c>
-      <c r="D10" t="n">
-        <v>2412.036478524168</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="C20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" t="n">
+        <v>5335.502558106416</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Respuesta por edad</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
         <is>
           <t>id_respuesta</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B24" s="1" t="inlineStr">
         <is>
           <t>Respuesta</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Hombre</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Mujer</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
+      <c r="C24" s="1" t="inlineStr">
+        <is>
+          <t>18-24</t>
+        </is>
+      </c>
+      <c r="D24" s="1" t="inlineStr">
+        <is>
+          <t>25-34</t>
+        </is>
+      </c>
+      <c r="E24" s="1" t="inlineStr">
+        <is>
+          <t>35-44</t>
+        </is>
+      </c>
+      <c r="F24" s="1" t="inlineStr">
+        <is>
+          <t>45-54</t>
+        </is>
+      </c>
+      <c r="G24" s="1" t="inlineStr">
+        <is>
+          <t>55-64</t>
+        </is>
+      </c>
+      <c r="H24" s="1" t="inlineStr">
+        <is>
+          <t>65-74</t>
+        </is>
+      </c>
+      <c r="I24" s="1" t="inlineStr">
+        <is>
+          <t>75 o mas</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Presencial</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>1478124.922820756</v>
-      </c>
-      <c r="D2" t="n">
-        <v>609330.4622021738</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Usted principalmente</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>216317.3016169026</v>
+      </c>
+      <c r="D25" t="n">
+        <v>376948.7731661667</v>
+      </c>
+      <c r="E25" t="n">
+        <v>408160.7543088065</v>
+      </c>
+      <c r="F25" t="n">
+        <v>294392.235259081</v>
+      </c>
+      <c r="G25" t="n">
+        <v>227253.3219970999</v>
+      </c>
+      <c r="H25" t="n">
+        <v>152161.0457217082</v>
+      </c>
+      <c r="I25" t="n">
+        <v>84023.78115182888</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Híbrido</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>38294.98199408736</v>
-      </c>
-      <c r="D3" t="n">
-        <v>54596.0112292008</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Usted y otra(s) persona(s) del hogar por igual</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>482274.1399185352</v>
+      </c>
+      <c r="D26" t="n">
+        <v>427269.4914949934</v>
+      </c>
+      <c r="E26" t="n">
+        <v>388247.2145975914</v>
+      </c>
+      <c r="F26" t="n">
+        <v>215822.7846575707</v>
+      </c>
+      <c r="G26" t="n">
+        <v>193808.6636886268</v>
+      </c>
+      <c r="H26" t="n">
+        <v>160333.6596818079</v>
+      </c>
+      <c r="I26" t="n">
+        <v>71962.47887312061</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>A distancia / en casa</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>37784.16104675323</v>
-      </c>
-      <c r="D4" t="n">
-        <v>46342.3751314176</v>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Otro(a) miembro del hogar</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>146579.5703655435</v>
+      </c>
+      <c r="D27" t="n">
+        <v>162037.2098215213</v>
+      </c>
+      <c r="E27" t="n">
+        <v>177690.4070462451</v>
+      </c>
+      <c r="F27" t="n">
+        <v>119939.0254338338</v>
+      </c>
+      <c r="G27" t="n">
+        <v>80997.93611449191</v>
+      </c>
+      <c r="H27" t="n">
+        <v>56755.18922419515</v>
+      </c>
+      <c r="I27" t="n">
+        <v>32172.73067049293</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>4</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Una persona contratada (vive o no en el hogar)</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>23131.79189647724</v>
+      </c>
+      <c r="D28" t="n">
+        <v>20965.95172470788</v>
+      </c>
+      <c r="E28" t="n">
+        <v>18283.08605914807</v>
+      </c>
+      <c r="F28" t="n">
+        <v>18826.34476076039</v>
+      </c>
+      <c r="G28" t="n">
+        <v>22149.0848096203</v>
+      </c>
+      <c r="H28" t="n">
+        <v>21140.3448870139</v>
+      </c>
+      <c r="I28" t="n">
+        <v>9337.969300189559</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>5</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Usted, con ayuda de una persona contratada uno o más días a la semana</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>145.5433803417732</v>
+      </c>
+      <c r="D29" t="n">
+        <v>508.6826462657611</v>
+      </c>
+      <c r="E29" t="n">
+        <v>311.2078410756614</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" t="n">
+        <v>3986.175719403531</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" t="n">
+        <v>460.113862108209</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>6</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Otro miembro del hogar, con ayuda de una persona contratada uno o más días a la semana</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" t="n">
+        <v>145.5433803417732</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" t="n">
+        <v>333.6691996024315</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>9999</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>No contesta</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" t="n">
+        <v>5335.502558106416</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>